<commit_message>
Add Wyckoff phase analyzer + integrated Excel with phase-based batch entry plan
Co-authored-by: a1944588323-MING <283437248+a1944588323-MING@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/stock_screener/资金分配可视化.xlsx
+++ b/stock_screener/资金分配可视化.xlsx
@@ -10,7 +10,8 @@
     <sheet name="📊 总览" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="🇺🇸 美股 AI 能源" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="🇨🇳 A股 存储与AI" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="⚡ 信号汇总" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="🌊 Wyckoff 详细" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="⚡ 操作信号" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,8 +25,8 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;%&quot;"/>
-    <numFmt numFmtId="168" formatCode="+0.0%;-0.0%"/>
-    <numFmt numFmtId="169" formatCode="&quot;¥&quot;#,##0"/>
+    <numFmt numFmtId="168" formatCode="&quot;¥&quot;#,##0"/>
+    <numFmt numFmtId="169" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -55,6 +56,7 @@
     </font>
     <font>
       <name val="微软雅黑"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -80,7 +82,8 @@
     <font>
       <name val="微软雅黑"/>
       <b val="1"/>
-      <sz val="11"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -141,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,13 +152,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,11 +170,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -182,43 +188,36 @@
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFE6E6"/>
-          <bgColor rgb="00FFE6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -232,6 +231,22 @@
         <patternFill patternType="solid">
           <fgColor rgb="00E2EFDA"/>
           <bgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+          <bgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFE6E6"/>
+          <bgColor rgb="00FFE6E6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -320,7 +335,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>美股 AI 能源 (8 只) - 资金分配比例</a:t>
+              <a:t>美股 AI 能源 (8 只) - 首批资金分配</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -334,7 +349,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🇺🇸 美股 AI 能源'!D4</f>
+              <f>'🇺🇸 美股 AI 能源'!O4</f>
             </strRef>
           </tx>
           <spPr>
@@ -349,7 +364,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'🇺🇸 美股 AI 能源'!$D$5:$D$12</f>
+              <f>'🇺🇸 美股 AI 能源'!$O$5:$O$12</f>
             </numRef>
           </val>
         </ser>
@@ -382,7 +397,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>综合评分排序</a:t>
+              <a:t>Wyckoff 首批仓位 %</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -397,7 +412,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🇺🇸 美股 AI 能源'!C4</f>
+              <f>'🇺🇸 美股 AI 能源'!N4</f>
             </strRef>
           </tx>
           <spPr>
@@ -412,7 +427,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'🇺🇸 美股 AI 能源'!$C$5:$C$12</f>
+              <f>'🇺🇸 美股 AI 能源'!$N$5:$N$12</f>
             </numRef>
           </val>
         </ser>
@@ -429,21 +444,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>综合分</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -456,21 +456,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>股票</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -497,7 +482,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>A 股 存储/AI (4 只) - 资金分配比例</a:t>
+              <a:t>A 股 存储 AI (4 只) - 首批资金分配</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -511,7 +496,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🇨🇳 A股 存储与AI'!D4</f>
+              <f>'🇨🇳 A股 存储与AI'!O4</f>
             </strRef>
           </tx>
           <spPr>
@@ -526,7 +511,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'🇨🇳 A股 存储与AI'!$D$5:$D$8</f>
+              <f>'🇨🇳 A股 存储与AI'!$O$5:$O$8</f>
             </numRef>
           </val>
         </ser>
@@ -559,7 +544,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>综合评分排序</a:t>
+              <a:t>Wyckoff 首批仓位 %</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -574,7 +559,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🇨🇳 A股 存储与AI'!C4</f>
+              <f>'🇨🇳 A股 存储与AI'!N4</f>
             </strRef>
           </tx>
           <spPr>
@@ -589,7 +574,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'🇨🇳 A股 存储与AI'!$C$5:$C$8</f>
+              <f>'🇨🇳 A股 存储与AI'!$N$5:$N$8</f>
             </numRef>
           </val>
         </ser>
@@ -606,21 +591,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>综合分</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -633,21 +603,6 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>股票</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -666,7 +621,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -688,7 +643,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>25</row>
       <rowOff>0</rowOff>
@@ -715,7 +670,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -737,7 +692,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>25</row>
       <rowOff>0</rowOff>
@@ -1049,24 +1004,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 资金分配 - 总览</t>
+          <t>📊 资金分配 + Wyckoff 形态分析 - 总览</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据来源: yfinance | 平均筹码代理: 60d VWAP | 主力推断: OBV+CMF+涨跌量比</t>
+          <t>数据来源: yfinance | Wyckoff 阶段: A/B/C/D/E (吸筹/派发) | 主力推断: OBV+CMF+涨跌量比</t>
         </is>
       </c>
     </row>
@@ -1083,17 +1038,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>总分</t>
+          <t>强建仓</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>首选(评分最高)</t>
+          <t>试探仓</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>投机仓(评分最低)</t>
+          <t>禁止建仓</t>
         </is>
       </c>
     </row>
@@ -1107,198 +1062,224 @@
         <v>8</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>334</v>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>EXE (80分)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>OKLO (18分)</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>🇨🇳 A 股 存储/AI</t>
+          <t>🇨🇳 A 股 存储 AI</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>111</v>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>603893.SS (48分)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>603690.SS (8分)</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>📋 评分维度说明</t>
+          <t>📚 Wyckoff 阶段说明</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>位置 % (52周区间)</t>
+          <t>吸筹周期 A 阶段(止跌)</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>&lt;10% +30 分,&lt;20% +25 分,&lt;30% +18 分,&gt;80% 0 分</t>
+          <t>长期下跌后初步止跌,价格停止创新低。⚠️ 还不能建仓</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>RSI 摆动</t>
+          <t>吸筹周期 B 阶段(吸筹震荡)</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>&lt;25 +15 分,&lt;35 +10 分,&gt;70 -10 分</t>
+          <t>横盘震荡,主力低位吸筹。🟡 可小仓位试探(20-30%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>PE (TTM)</t>
+          <t>吸筹周期 C 阶段(Spring 假跌破)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>&lt;15 +15 分,&lt;25 +10 分,&gt;50 -5 分,&gt;80 -10 分</t>
+          <t>短暂跌破前低后强力收回。✅ 最佳建仓点(60% 重仓)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>营收增长 YoY</t>
+          <t>吸筹周期 D 阶段(SOS 强势)</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>&gt;30% +15 分,&gt;15% +10 分,&lt;-10% -10 分</t>
+          <t>Sign of Strength,放量上涨突破。✅ 趋势确认建仓(70%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>利润率</t>
+          <t>吸筹周期 E 阶段(上升趋势)</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>&gt;20% +10 分,&lt;-5% -10 分</t>
+          <t>脱离吸筹区进入上升通道。🟢 已在趋势中,回踩加仓</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>ROE</t>
+          <t>派发周期 A 阶段(派发开始)</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>&gt;20% +10 分,&gt;10% +5 分,&lt;0 -5 分</t>
+          <t>高位放量但 OBV 走弱。🚫 不建仓</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>主力资金信号</t>
+          <t>派发周期 B 阶段(派发震荡)</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>建仓 +10 分,净流入 +5 分,派发 -10 分</t>
+          <t>高位横盘,主力派发。🚫 不建仓</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>市值规避微盘</t>
+          <t>派发周期 C 阶段(UTAD 假突破)</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>&lt;10亿 -5 分,&gt;500亿 +3 分</t>
+          <t>短暂突破前高后回落。🚫 顶部信号,远离</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>派发周期 D 阶段(SOW 弱势)</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Sign of Weakness,跌破支撑。🚫 等待跌至 MA200 再评估</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>派发周期 E 阶段(下跌趋势)</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>进入下降通道。🚫 等止跌信号</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>⚠️ 重要说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>1. 平均筹码价格 用 60 日 VWAP(成交量加权均价)代理 — 严格的'持仓成本'需要 Tick 数据,本表近似</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>2. 主力资金/庄家建仓 用 OBV+CMF+涨跌量比 推断 — 准确判断需要 L2 主力净流入数据</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>3. 本报告为按规则的资金分配,不构成任何投资建议。投资决策请结合基本面、行业景气度自行判断</t>
+          <t>1. Wyckoff 阶段判断结合: 52W 位置 + MA200/MA60 趋势 + 振幅收敛 + OBV + Spring/UTAD 检测</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>4. 风险提示: 单笔仓位 ≥ 5%, ≤ 25%(4只组合 ≤ 40%);跌破 52W 低 5% 强制止损</t>
+          <t>2. 平均筹码价格 用 60 日 VWAP 代理 — 严格的'持仓成本'需要 Tick 数据,本表近似</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>3. 主力资金/庄家 用 OBV+CMF+涨跌量比 推断 — 准确判断需要 L2 主力净流入数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>4. 本报告为按规则的资金分配,不构成任何投资建议</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>5. 风险提示: 跌破止损位强制止损,Spring 失败立即清仓</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="19">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="B16:E16"/>
     <mergeCell ref="A21:E21"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="B18:E18"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="A8:E8"/>
     <mergeCell ref="B10:E10"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1310,38 +1291,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>💰 美股 AI 能源 (8 只) 资金分配方案</t>
+          <t>💰 美股 AI 能源 (8 只) - 资金分配 + Wyckoff 形态</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>总资金 $100,000 | 数据时间: 实时(yfinance)</t>
+          <t>总资金 $100,000 | 首批仓位按 Wyckoff 阶段调整</t>
         </is>
       </c>
     </row>
@@ -1368,12 +1350,12 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>分配金额</t>
+          <t>理论金额</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>估算手数</t>
+          <t>股价</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
@@ -1408,22 +1390,27 @@
       </c>
       <c r="M4" s="11" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>Wyckoff 阶段</t>
         </is>
       </c>
       <c r="N4" s="11" t="inlineStr">
         <is>
-          <t>60d VWAP</t>
+          <t>首批 %</t>
         </is>
       </c>
       <c r="O4" s="11" t="inlineStr">
         <is>
-          <t>当前/VWAP</t>
+          <t>首批金额</t>
         </is>
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
-          <t>主力推断</t>
+          <t>第二批触发</t>
+        </is>
+      </c>
+      <c r="Q4" s="11" t="inlineStr">
+        <is>
+          <t>止损</t>
         </is>
       </c>
     </row>
@@ -1433,54 +1420,59 @@
           <t>EXE</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Expand Energy Corporation</t>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Expand Energy Corporat</t>
         </is>
       </c>
       <c r="C5" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.2395209580838323</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="15" t="n">
         <v>23952.09580838323</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>251</v>
-      </c>
-      <c r="G5" s="15" t="n">
-        <v>22788939776</v>
-      </c>
-      <c r="H5" s="16" t="n">
-        <v>7.087798</v>
-      </c>
-      <c r="I5" s="13" t="n">
+        <v>95.31999999999999</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>22803294208</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <v>7.0922623</v>
+      </c>
+      <c r="I5" s="14" t="n">
         <v>0.41</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="14" t="n">
         <v>0.24906999</v>
       </c>
-      <c r="K5" s="13" t="n">
+      <c r="K5" s="14" t="n">
         <v>0.17568001</v>
       </c>
-      <c r="L5" s="17" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="M5" s="16" t="n">
-        <v>38.9</v>
-      </c>
-      <c r="N5" s="18" t="n">
-        <v>103.57</v>
-      </c>
-      <c r="O5" s="19" t="n">
-        <v>-0.08019999999999999</v>
-      </c>
-      <c r="P5" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="L5" s="18" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="N5" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O5" s="15" t="n">
+        <v>14371.25748502994</v>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>突破 100.09(+5%) 加仓</t>
+        </is>
+      </c>
+      <c r="Q5" s="20" t="n">
+        <v>94.37</v>
       </c>
     </row>
     <row r="6">
@@ -1489,7 +1481,7 @@
           <t>VST</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Vistra Corp.</t>
         </is>
@@ -1497,46 +1489,51 @@
       <c r="C6" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>0.1796407185628743</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="15" t="n">
         <v>17964.07185628742</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>126</v>
-      </c>
-      <c r="G6" s="15" t="n">
-        <v>47987810304</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>23.799332</v>
-      </c>
-      <c r="I6" s="13" t="n">
+        <v>142.69</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>48112566272</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>23.861204</v>
+      </c>
+      <c r="I6" s="14" t="n">
         <v>0.434</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="14" t="n">
         <v>0.11525</v>
       </c>
-      <c r="K6" s="13" t="n">
+      <c r="K6" s="14" t="n">
         <v>0.42898</v>
       </c>
-      <c r="L6" s="17" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="M6" s="16" t="n">
-        <v>37.1</v>
-      </c>
-      <c r="N6" s="18" t="n">
-        <v>159.54</v>
-      </c>
-      <c r="O6" s="19" t="n">
-        <v>-0.1079</v>
-      </c>
-      <c r="P6" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
+      <c r="L6" s="18" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>A (止跌)</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O6" s="15" t="n">
+        <v>2694.610778443114</v>
+      </c>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 173.54(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="Q6" s="20" t="n">
+        <v>131.27</v>
       </c>
     </row>
     <row r="7">
@@ -1545,54 +1542,59 @@
           <t>PEG</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Public Service Enterprise</t>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Public Service Enterpr</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
         <v>53</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.1586826347305389</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="15" t="n">
         <v>15868.26347305389</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>206</v>
-      </c>
-      <c r="G7" s="15" t="n">
-        <v>38241185792</v>
-      </c>
-      <c r="H7" s="16" t="n">
-        <v>16.977875</v>
-      </c>
-      <c r="I7" s="13" t="n">
+        <v>77.12</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>38430547968</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>17.061947</v>
+      </c>
+      <c r="I7" s="14" t="n">
         <v>0.194</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="14" t="n">
         <v>0.17688</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K7" s="14" t="n">
         <v>0.13441</v>
       </c>
-      <c r="L7" s="17" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="M7" s="16" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="N7" s="18" t="n">
-        <v>81.65000000000001</v>
-      </c>
-      <c r="O7" s="19" t="n">
-        <v>-0.0602</v>
-      </c>
-      <c r="P7" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="L7" s="18" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>B (吸筹震荡)</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O7" s="15" t="n">
+        <v>4760.479041916167</v>
+      </c>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>突破 83.82 加 / 回踩 76.60 不破再加</t>
+        </is>
+      </c>
+      <c r="Q7" s="20" t="n">
+        <v>71.23999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -1601,54 +1603,59 @@
           <t>CEG</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Constellation Energy Corp</t>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Constellation Energy C</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
         <v>51</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>0.1526946107784431</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <v>15269.46107784431</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>55</v>
-      </c>
-      <c r="G8" s="15" t="n">
-        <v>99971989504</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <v>24.04735</v>
-      </c>
-      <c r="I8" s="13" t="n">
+        <v>277.11</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>100085768192</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>24.074718</v>
+      </c>
+      <c r="I8" s="14" t="n">
         <v>0.638</v>
       </c>
-      <c r="J8" s="13" t="n">
+      <c r="J8" s="14" t="n">
         <v>0.12693</v>
       </c>
-      <c r="K8" s="13" t="n">
+      <c r="K8" s="14" t="n">
         <v>0.16104999</v>
       </c>
-      <c r="L8" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="M8" s="16" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="N8" s="18" t="n">
-        <v>301.37</v>
-      </c>
-      <c r="O8" s="19" t="n">
-        <v>-0.08160000000000001</v>
-      </c>
-      <c r="P8" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
+      <c r="L8" s="18" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>A-&gt;B (筑底)</t>
+        </is>
+      </c>
+      <c r="N8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O8" s="15" t="n">
+        <v>2290.419161676647</v>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 338.66(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="Q8" s="20" t="n">
+        <v>254.93</v>
       </c>
     </row>
     <row r="9">
@@ -1657,7 +1664,7 @@
           <t>NRG</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>NRG Energy, Inc.</t>
         </is>
@@ -1665,46 +1672,51 @@
       <c r="C9" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>0.08083832335329341</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="15" t="n">
         <v>8083.832335329341</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>61</v>
-      </c>
-      <c r="G9" s="15" t="n">
-        <v>27747885056</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>144.52197</v>
-      </c>
-      <c r="I9" s="13" t="n">
+        <v>131.46</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>27737333760</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>144.46703</v>
+      </c>
+      <c r="I9" s="14" t="n">
         <v>0.195</v>
       </c>
-      <c r="J9" s="13" t="n">
+      <c r="J9" s="14" t="n">
         <v>0.00738</v>
       </c>
-      <c r="K9" s="13" t="n">
+      <c r="K9" s="14" t="n">
         <v>0.062480003</v>
       </c>
-      <c r="L9" s="17" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="M9" s="16" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="N9" s="18" t="n">
-        <v>157.33</v>
-      </c>
-      <c r="O9" s="19" t="n">
-        <v>-0.1641</v>
-      </c>
-      <c r="P9" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
+      <c r="L9" s="18" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>A/B (筑底中)</t>
+        </is>
+      </c>
+      <c r="N9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O9" s="15" t="n">
+        <v>1212.574850299401</v>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 180.23(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="Q9" s="20" t="n">
+        <v>120.95</v>
       </c>
     </row>
     <row r="10">
@@ -1713,7 +1725,7 @@
           <t>STEM</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Stem, Inc.</t>
         </is>
@@ -1721,42 +1733,47 @@
       <c r="C10" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>0.0748502994011976</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="15" t="n">
         <v>7485.02994011976</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>836</v>
-      </c>
-      <c r="G10" s="15" t="n">
-        <v>80164728</v>
-      </c>
-      <c r="H10" s="16" t="n"/>
-      <c r="I10" s="13" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>80127112</v>
+      </c>
+      <c r="H10" s="17" t="n"/>
+      <c r="I10" s="14" t="n">
         <v>-0.108</v>
       </c>
-      <c r="J10" s="13" t="n">
+      <c r="J10" s="14" t="n">
         <v>0.94162005</v>
       </c>
-      <c r="K10" s="13" t="n"/>
-      <c r="L10" s="17" t="n">
+      <c r="K10" s="14" t="n"/>
+      <c r="L10" s="18" t="n">
         <v>11.5</v>
       </c>
-      <c r="M10" s="16" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="N10" s="18" t="n">
-        <v>10.52</v>
-      </c>
-      <c r="O10" s="19" t="n">
-        <v>-0.1492</v>
-      </c>
-      <c r="P10" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>A/B (筑底中)</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O10" s="15" t="n">
+        <v>1122.754491017964</v>
+      </c>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 12.64(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="Q10" s="20" t="n">
+        <v>8.23</v>
       </c>
     </row>
     <row r="11">
@@ -1765,52 +1782,57 @@
           <t>SMR</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>NuScale Power Corporation</t>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>NuScale Power Corporat</t>
         </is>
       </c>
       <c r="C11" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>0.05988023952095808</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="15" t="n">
         <v>5988.023952095808</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>482</v>
-      </c>
-      <c r="G11" s="15" t="n">
-        <v>4292784640</v>
-      </c>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="13" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>4239795968</v>
+      </c>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="14" t="n">
         <v>-0.958</v>
       </c>
-      <c r="J11" s="13" t="n">
+      <c r="J11" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="13" t="n">
+      <c r="K11" s="14" t="n">
         <v>-0.8305</v>
       </c>
-      <c r="L11" s="17" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="M11" s="16" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="N11" s="18" t="n">
-        <v>11.98</v>
-      </c>
-      <c r="O11" s="19" t="n">
-        <v>0.0354</v>
-      </c>
-      <c r="P11" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="L11" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="N11" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O11" s="15" t="n">
+        <v>3592.814371257485</v>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>突破 12.86(+5%) 加仓</t>
+        </is>
+      </c>
+      <c r="Q11" s="20" t="n">
+        <v>9.369999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1819,7 +1841,7 @@
           <t>OKLO</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Oklo Inc.</t>
         </is>
@@ -1827,42 +1849,47 @@
       <c r="C12" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>0.05389221556886228</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <v>5389.221556886228</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>75</v>
-      </c>
-      <c r="G12" s="15" t="n">
-        <v>12417876992</v>
-      </c>
-      <c r="H12" s="16" t="n"/>
-      <c r="I12" s="13" t="n"/>
-      <c r="J12" s="13" t="n">
+        <v>70.76000000000001</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>12306568192</v>
+      </c>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="14" t="n"/>
+      <c r="J12" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="13" t="n">
+      <c r="K12" s="14" t="n">
         <v>-0.12236</v>
       </c>
-      <c r="L12" s="17" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="M12" s="16" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N12" s="18" t="n">
-        <v>64.56</v>
-      </c>
-      <c r="O12" s="19" t="n">
-        <v>0.1059</v>
-      </c>
-      <c r="P12" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="L12" s="18" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>B (吸筹震荡)</t>
+        </is>
+      </c>
+      <c r="N12" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O12" s="15" t="n">
+        <v>1616.766467065868</v>
+      </c>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>突破 83.13 加 / 回踩 60.81 不破再加</t>
+        </is>
+      </c>
+      <c r="Q12" s="20" t="n">
+        <v>56.55</v>
       </c>
     </row>
     <row r="14">
@@ -1890,13 +1917,30 @@
       <c r="L14" s="21" t="n"/>
       <c r="M14" s="21" t="n"/>
       <c r="N14" s="21" t="n"/>
-      <c r="O14" s="21" t="n"/>
+      <c r="O14" s="23">
+        <f>SUM(O5:O12)</f>
+        <v/>
+      </c>
       <c r="P14" s="21" t="n"/>
+      <c r="Q14" s="21" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>说明:</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>理论金额=综合分加权;首批金额=理论金额×Wyckoff首批比例;余下资金等第二批触发条件</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+  <mergeCells count="3">
+    <mergeCell ref="B16:Q16"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:C12">
     <cfRule type="colorScale" priority="1">
@@ -1976,39 +2020,39 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M12">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="20"/>
-        <cfvo type="num" val="50"/>
-        <cfvo type="num" val="80"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
+  <conditionalFormatting sqref="N5:N12">
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="0000B050"/>
+      </dataBar>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O12">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="num" val="-0.2"/>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.2"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0000B050"/>
+      </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P12">
+  <conditionalFormatting sqref="A5:Q12">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>ISNUMBER(SEARCH("派发",P5))</formula>
+      <formula>ISNUMBER(SEARCH("Spring",$M5))</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="1">
-      <formula>ISNUMBER(SEARCH("建仓",P5))</formula>
+      <formula>ISNUMBER(SEARCH("SOS",$M5))</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="2">
-      <formula>ISNUMBER(SEARCH("流入",P5))</formula>
+    <cfRule type="expression" priority="12" dxfId="1">
+      <formula>ISNUMBER(SEARCH("E (",$M5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="2">
+      <formula>ISNUMBER(SEARCH("吸筹",$M5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="3">
+      <formula>OR(ISNUMBER(SEARCH("UTAD",$M5)),ISNUMBER(SEARCH("派发",$M5)),ISNUMBER(SEARCH("SOW",$M5)),ISNUMBER(SEARCH("顶部",$M5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2022,38 +2066,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>💰 A 股 存储/AI (4 只) 资金分配方案</t>
+          <t>💰 A 股 存储 AI (4 只) - 资金分配 + Wyckoff 形态</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>总资金 ¥100,000 | 数据时间: 实时(yfinance)</t>
+          <t>总资金 ¥100,000 | 首批仓位按 Wyckoff 阶段调整</t>
         </is>
       </c>
     </row>
@@ -2080,12 +2125,12 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>分配金额</t>
+          <t>理论金额</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>估算手数</t>
+          <t>股价</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
@@ -2120,22 +2165,27 @@
       </c>
       <c r="M4" s="11" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>Wyckoff 阶段</t>
         </is>
       </c>
       <c r="N4" s="11" t="inlineStr">
         <is>
-          <t>60d VWAP</t>
+          <t>首批 %</t>
         </is>
       </c>
       <c r="O4" s="11" t="inlineStr">
         <is>
-          <t>当前/VWAP</t>
+          <t>首批金额</t>
         </is>
       </c>
       <c r="P4" s="11" t="inlineStr">
         <is>
-          <t>主力推断</t>
+          <t>第二批触发</t>
+        </is>
+      </c>
+      <c r="Q4" s="11" t="inlineStr">
+        <is>
+          <t>止损</t>
         </is>
       </c>
     </row>
@@ -2145,54 +2195,59 @@
           <t>603893.SS</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Rockchip Electronics Co.,</t>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Rockchip Electronics C</t>
         </is>
       </c>
       <c r="C5" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.4</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="25" t="n">
         <v>40000</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>222</v>
-      </c>
-      <c r="G5" s="15" t="n">
+        <v>179.43</v>
+      </c>
+      <c r="G5" s="16" t="n">
         <v>76014780416</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <v>65.65818</v>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="14" t="n">
         <v>0.362</v>
       </c>
-      <c r="J5" s="13" t="n">
+      <c r="J5" s="14" t="n">
         <v>0.24555999</v>
       </c>
-      <c r="K5" s="13" t="n">
+      <c r="K5" s="14" t="n">
         <v>0.27346</v>
       </c>
-      <c r="L5" s="17" t="n">
+      <c r="L5" s="18" t="n">
         <v>36.4</v>
       </c>
-      <c r="M5" s="16" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="N5" s="18" t="n">
-        <v>172.32</v>
-      </c>
-      <c r="O5" s="19" t="n">
-        <v>0.0413</v>
-      </c>
-      <c r="P5" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>中位震荡</t>
+        </is>
+      </c>
+      <c r="N5" s="19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O5" s="25" t="n">
+        <v>8000</v>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t>无明确方向</t>
+        </is>
+      </c>
+      <c r="Q5" s="20" t="n">
+        <v>165.08</v>
       </c>
     </row>
     <row r="6">
@@ -2201,7 +2256,7 @@
           <t>002230.SZ</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>iFLYTEK CO.,LTD</t>
         </is>
@@ -2209,46 +2264,51 @@
       <c r="C6" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>0.2769230769230769</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="25" t="n">
         <v>27692.3076923077</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>567</v>
-      </c>
-      <c r="G6" s="15" t="n">
+        <v>48.83</v>
+      </c>
+      <c r="G6" s="16" t="n">
         <v>118662742016</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>133.51352</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I6" s="14" t="n">
         <v>0.132</v>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="J6" s="14" t="n">
         <v>0.03113</v>
       </c>
-      <c r="K6" s="13" t="n">
+      <c r="K6" s="14" t="n">
         <v>0.04538</v>
       </c>
-      <c r="L6" s="17" t="n">
+      <c r="L6" s="18" t="n">
         <v>17.3</v>
       </c>
-      <c r="M6" s="16" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="N6" s="18" t="n">
-        <v>51.5</v>
-      </c>
-      <c r="O6" s="19" t="n">
-        <v>-0.0519</v>
-      </c>
-      <c r="P6" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>C-&gt;D (Spring 已确认)</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="O6" s="25" t="n">
+        <v>19384.61538461539</v>
+      </c>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>突破 50.29(+3%) 加仓</t>
+        </is>
+      </c>
+      <c r="Q6" s="20" t="n">
+        <v>49.17</v>
       </c>
     </row>
     <row r="7">
@@ -2257,54 +2317,59 @@
           <t>603160.SS</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Shenzhen Goodix Technolog</t>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Shenzhen Goodix Techno</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.2341880341880342</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="25" t="n">
         <v>23418.80341880342</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>352</v>
-      </c>
-      <c r="G7" s="15" t="n">
+        <v>66.37</v>
+      </c>
+      <c r="G7" s="16" t="n">
         <v>31601100800</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <v>41.359756</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="14" t="n">
         <v>-0.09</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J7" s="14" t="n">
         <v>0.16354999</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K7" s="14" t="n">
         <v>0.082720004</v>
       </c>
-      <c r="L7" s="17" t="n">
+      <c r="L7" s="18" t="n">
         <v>13.4</v>
       </c>
-      <c r="M7" s="16" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="N7" s="18" t="n">
-        <v>70.3</v>
-      </c>
-      <c r="O7" s="19" t="n">
-        <v>-0.05599999999999999</v>
-      </c>
-      <c r="P7" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O7" s="25" t="n">
+        <v>14051.28205128205</v>
+      </c>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>突破 69.69(+5%) 加仓</t>
+        </is>
+      </c>
+      <c r="Q7" s="20" t="n">
+        <v>62.45</v>
       </c>
     </row>
     <row r="8">
@@ -2313,52 +2378,57 @@
           <t>603690.SS</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PNC Process Systems Co., </t>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>PNC Process Systems Co</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>0.08888888888888889</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="25" t="n">
         <v>8888.888888888889</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>330</v>
-      </c>
-      <c r="G8" s="15" t="n">
+        <v>26.87</v>
+      </c>
+      <c r="G8" s="16" t="n">
         <v>10539176960</v>
       </c>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="13" t="n">
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="14" t="n">
         <v>-0.317</v>
       </c>
-      <c r="J8" s="13" t="n">
+      <c r="J8" s="14" t="n">
         <v>-0.02538</v>
       </c>
-      <c r="K8" s="13" t="n">
+      <c r="K8" s="14" t="n">
         <v>-0.03528</v>
       </c>
-      <c r="L8" s="17" t="n">
+      <c r="L8" s="18" t="n">
         <v>20.3</v>
       </c>
-      <c r="M8" s="16" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="N8" s="18" t="n">
-        <v>26.28</v>
-      </c>
-      <c r="O8" s="19" t="n">
-        <v>0.0223</v>
-      </c>
-      <c r="P8" s="20" t="inlineStr">
-        <is>
-          <t>✅ 资金温和净流入</t>
-        </is>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>C-&gt;D (Spring 已确认)</t>
+        </is>
+      </c>
+      <c r="N8" s="19" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="O8" s="25" t="n">
+        <v>6222.222222222222</v>
+      </c>
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t>突破 27.68(+3%) 加仓</t>
+        </is>
+      </c>
+      <c r="Q8" s="20" t="n">
+        <v>25.4</v>
       </c>
     </row>
     <row r="10">
@@ -2373,7 +2443,7 @@
         <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="26">
         <f>SUM(E5:E8)</f>
         <v/>
       </c>
@@ -2386,13 +2456,30 @@
       <c r="L10" s="21" t="n"/>
       <c r="M10" s="21" t="n"/>
       <c r="N10" s="21" t="n"/>
-      <c r="O10" s="21" t="n"/>
+      <c r="O10" s="26">
+        <f>SUM(O5:O8)</f>
+        <v/>
+      </c>
       <c r="P10" s="21" t="n"/>
+      <c r="Q10" s="21" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>说明:</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>理论金额=综合分加权;首批金额=理论金额×Wyckoff首批比例;余下资金等第二批触发条件</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="B12:Q12"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="C5:C8">
     <cfRule type="colorScale" priority="1">
@@ -2472,39 +2559,39 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M8">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="num" val="20"/>
-        <cfvo type="num" val="50"/>
-        <cfvo type="num" val="80"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
+  <conditionalFormatting sqref="N5:N8">
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="0000B050"/>
+      </dataBar>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O8">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="num" val="-0.2"/>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.2"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFFFFF"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0000B050"/>
+      </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P8">
+  <conditionalFormatting sqref="A5:Q8">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>ISNUMBER(SEARCH("派发",P5))</formula>
+      <formula>ISNUMBER(SEARCH("Spring",$M5))</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="1">
-      <formula>ISNUMBER(SEARCH("建仓",P5))</formula>
+      <formula>ISNUMBER(SEARCH("SOS",$M5))</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="2">
-      <formula>ISNUMBER(SEARCH("流入",P5))</formula>
+    <cfRule type="expression" priority="12" dxfId="1">
+      <formula>ISNUMBER(SEARCH("E (",$M5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="2">
+      <formula>ISNUMBER(SEARCH("吸筹",$M5))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="3">
+      <formula>OR(ISNUMBER(SEARCH("UTAD",$M5)),ISNUMBER(SEARCH("派发",$M5)),ISNUMBER(SEARCH("SOW",$M5)),ISNUMBER(SEARCH("顶部",$M5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2518,21 +2605,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚡ 主力资金信号 + 筹码状态</t>
+          <t>🌊 Wyckoff 形态详细分析(12 只)</t>
         </is>
       </c>
     </row>
@@ -2554,417 +2650,1425 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>筹码状态</t>
+          <t>周期</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>主力推断</t>
+          <t>Wyckoff 阶段</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
+          <t>形态详情</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>可信度</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>位置 %</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>MA60 斜率</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>振幅比</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>OBV变化</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>涨跌量比</t>
+        </is>
+      </c>
+      <c r="M3" s="11" t="inlineStr">
+        <is>
+          <t>Spring/UTAD</t>
+        </is>
+      </c>
+      <c r="N3" s="11" t="inlineStr">
+        <is>
           <t>操作建议</t>
         </is>
       </c>
+      <c r="O3" s="11" t="inlineStr">
+        <is>
+          <t>首批 %</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>EXE</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
-        <is>
-          <t>Expand Energy Corporation</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Expand Energy Corporat</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>刚出现 Spring 假跌破 (97.29),最佳建仓点之一</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="I4" s="27" t="n">
+        <v>-2.89</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>-1.613</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>Spring @ 97.29</t>
+        </is>
+      </c>
+      <c r="N4" s="13" t="inlineStr">
+        <is>
+          <t>✅ 强烈建仓</t>
+        </is>
+      </c>
+      <c r="O4" s="19" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>VST</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Vistra Corp.</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E5" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
-      </c>
-      <c r="F5" s="20" t="inlineStr">
-        <is>
-          <t>🔴 警惕! 首笔不超过分配额 30%,等回调</t>
-        </is>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>A (止跌)</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>长跌后初步止跌,但还未确认企稳</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="I5" s="27" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="O5" s="19" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>PEG</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
-        <is>
-          <t>Public Service Enterprise</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Public Service Enterpr</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>B (吸筹震荡)</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>底部震荡,有吸筹特征</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="I6" s="27" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>-0.131</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>🟡 小仓位试探</t>
+        </is>
+      </c>
+      <c r="O6" s="19" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>CEG</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Constellation Energy Corp</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Constellation Energy C</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>🔴 警惕! 首笔不超过分配额 30%,等回调</t>
-        </is>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>A-&gt;B (筑底)</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>脱离极低位但未确认突破</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>-0.8139999999999999</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="O7" s="19" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>NRG</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>NRG Energy, Inc.</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>🔴 警惕! 首笔不超过分配额 30%,等回调</t>
-        </is>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>A/B (筑底中)</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>底部区域,但形态还不明朗</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I8" s="27" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <v>-0.263</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="O8" s="19" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>STEM</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Stem, Inc.</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>A/B (筑底中)</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>底部区域,但形态还不明朗</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="I9" s="27" t="n">
+        <v>-11.77</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="O9" s="19" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>SMR</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
-        <is>
-          <t>NuScale Power Corporation</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>NuScale Power Corporat</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>成本附近震荡</t>
-        </is>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>刚出现 Spring 假跌破 (9.65),最佳建仓点之一</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="27" t="n">
+        <v>-11.65</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>-1.891</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>Spring @ 9.65</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>✅ 强烈建仓</t>
+        </is>
+      </c>
+      <c r="O10" s="19" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>OKLO</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Oklo Inc.</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>🇺🇸 美股</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>套利盘多(price &gt; 60d VWAP +5%)</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F11" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>B (吸筹震荡)</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>底部震荡,有吸筹特征</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I11" s="27" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>🟡 小仓位试探</t>
+        </is>
+      </c>
+      <c r="O11" s="19" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>603893.SS</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>Rockchip Electronics Co.,</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Rockchip Electronics C</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>🇨🇳 A 股</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>成本附近震荡</t>
-        </is>
-      </c>
-      <c r="E12" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>中位震荡</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>无明确方向</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="I12" s="27" t="n">
+        <v>-2.42</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="13" t="inlineStr">
+        <is>
+          <t>⚪ 观望</t>
+        </is>
+      </c>
+      <c r="O12" s="19" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>002230.SZ</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>iFLYTEK CO.,LTD</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>🇨🇳 A 股</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>➖ 量价中性</t>
-        </is>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>⚪ 量价无明显方向,按计划执行</t>
-        </is>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>C-&gt;D (Spring 已确认)</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Spring 后已回升,SOS 信号待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="I13" s="27" t="n">
+        <v>-6.03</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>Spring @ 45.36</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>✅ 趋势确认建仓</t>
+        </is>
+      </c>
+      <c r="O13" s="19" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>603160.SS</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
-        <is>
-          <t>Shenzhen Goodix Technolog</t>
-        </is>
-      </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Shenzhen Goodix Techno</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>🇨🇳 A 股</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>深套(price &lt; 60d VWAP -5%)</t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>🔻 放量下跌 → 主力疑似派发</t>
-        </is>
-      </c>
-      <c r="F14" s="20" t="inlineStr">
-        <is>
-          <t>🔴 警惕! 首笔不超过分配额 30%,等回调</t>
-        </is>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>刚出现 Spring 假跌破 (64.38),最佳建仓点之一</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="I14" s="27" t="n">
+        <v>-6.22</v>
+      </c>
+      <c r="J14" s="12" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="K14" s="12" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>Spring @ 64.38</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>✅ 强烈建仓</t>
+        </is>
+      </c>
+      <c r="O14" s="19" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>603690.SS</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PNC Process Systems Co., </t>
-        </is>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>PNC Process Systems Co</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>🇨🇳 A 股</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>成本附近震荡</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>✅ 资金温和净流入</t>
-        </is>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>🟢 资金温和买入 - 可正常配置</t>
-        </is>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>accumulation</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>C-&gt;D (Spring 已确认)</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Spring 后已回升,SOS 信号待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="I15" s="27" t="n">
+        <v>-6.58</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Spring @ 23.67</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>✅ 趋势确认建仓</t>
+        </is>
+      </c>
+      <c r="O15" s="19" t="n">
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A4:F15">
+  <conditionalFormatting sqref="A4:O15">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>ISNUMBER(SEARCH("派发",$E4))</formula>
+      <formula>ISNUMBER(SEARCH("Spring",$E4))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>ISNUMBER(SEARCH("建仓",$E4))</formula>
+      <formula>ISNUMBER(SEARCH("SOS",$E4))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="3">
+      <formula>OR(ISNUMBER(SEARCH("UTAD",$E4)),ISNUMBER(SEARCH("派发",$E4)),ISNUMBER(SEARCH("SOW",$E4)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>ISNUMBER(SEARCH("吸筹",$E4))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O4:O15">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="0000B050"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>⚡ 操作信号汇总(分批建仓策略)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>市场</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Wyckoff 阶段</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>建议操作</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>第二批触发条件</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>止损价</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>首批 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>EXE</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Expand Energy Corporat</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>✅ 强烈建仓</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>突破 100.09(+5%) 加仓</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>94.37</v>
+      </c>
+      <c r="H4" s="19" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>SMR</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>NuScale Power Corporat</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>✅ 强烈建仓</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>突破 12.86(+5%) 加仓</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PEG</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Public Service Enterpr</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>B (吸筹震荡)</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>🟡 小仓位试探</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>突破 83.82 加 / 回踩 76.60 不破再加</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>71.23999999999999</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>OKLO</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Oklo Inc.</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>B (吸筹震荡)</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>🟡 小仓位试探</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>突破 83.13 加 / 回踩 60.81 不破再加</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>56.55</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Vistra Corp.</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>A (止跌)</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 173.54(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>131.27</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Constellation Energy C</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>A-&gt;B (筑底)</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 338.66(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>254.93</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>NRG</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>NRG Energy, Inc.</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>A/B (筑底中)</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 180.23(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>120.95</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>STEM</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Stem, Inc.</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>🇺🇸 美股</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>A/B (筑底中)</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ 暂不建仓</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>等待突破 12.64(确认 SOS)再建主仓</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>8.23</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>002230.SZ</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>iFLYTEK CO.,LTD</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>🇨🇳 A 股</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>C-&gt;D (Spring 已确认)</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>✅ 趋势确认建仓</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>突破 50.29(+3%) 加仓</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>49.17</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>603690.SS</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>PNC Process Systems Co</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>🇨🇳 A 股</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>C-&gt;D (Spring 已确认)</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>✅ 趋势确认建仓</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>突破 27.68(+3%) 加仓</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="H13" s="19" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>603160.SS</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Shenzhen Goodix Techno</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>🇨🇳 A 股</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>C (Spring)</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>✅ 强烈建仓</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>突破 69.69(+5%) 加仓</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="n">
+        <v>62.45</v>
+      </c>
+      <c r="H14" s="19" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>603893.SS</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Rockchip Electronics C</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>🇨🇳 A 股</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>中位震荡</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>⚪ 观望</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>无明确方向</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>165.08</v>
+      </c>
+      <c r="H15" s="19" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A4:H15">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>ISNUMBER(SEARCH("强烈建仓",$E4))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>OR(ISNUMBER(SEARCH("趋势确认",$E4)),ISNUMBER(SEARCH("趋势中",$E4)))</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>ISNUMBER(SEARCH("流入",$E4))</formula>
+      <formula>ISNUMBER(SEARCH("试探",$E4))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>ISNUMBER(SEARCH("不建仓",$E4))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4:H15">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="0000B050"/>
+      </dataBar>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>